<commit_message>
Week 7 (Part 10 & Backend): Complete TALASH backend integration. Added composite_evaluator.py (weighted 0-100 scoring, Tier 1-4 classifier across 8 modules), email_drafter.py (missing-info detection, LLM personalized follow-up emails), pipeline_orchestrator.py (MasterPipeline integrating Parts 1-10), FastAPI backend (api/ with /health, /candidates, /candidates/{id}, /compare, /email/{id}, /upload endpoints), run_backend.py (Uvicorn launcher), test_backend_api.py (7/7 end-to-end API tests passing). All 43 candidates evaluated with composite scores and tier classifications.
</commit_message>
<xml_diff>
--- a/data/analysis/book_aggregates.xlsx
+++ b/data/analysis/book_aggregates.xlsx
@@ -546,7 +546,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Candidate 01_MUHAMMAD_SALMAN has no books listed in their CV.</t>
+          <t>Candidate MUHAMMAD SALMAN has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -600,7 +600,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Candidate 02_MUHAMMAD_SHAHWAZ has no books listed in their CV.</t>
+          <t>Candidate MUHAMMAD SHAHWAZ has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Candidate 03_NASIR_ALI_SHAH has no books listed in their CV.</t>
+          <t>Candidate Nasir Ali Shah has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Candidate 04_MUHAMMAD_FARRUKH has no books listed in their CV.</t>
+          <t>Candidate Muhammad Farrukh Qureshi has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -762,7 +762,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Candidate 05_MUHAMMAD_MAJID has no books listed in their CV.</t>
+          <t>Candidate MUHAMMAD MAJID has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Candidate 06_FARMAN_ALI has no books listed in their CV.</t>
+          <t>Candidate Farman Ali has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Candidate 07_FIZA_MURTAZA has no books listed in their CV.</t>
+          <t>Candidate Fiza Murtaza has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -924,7 +924,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Candidate 08_TAYYABA_GULL has no books listed in their CV.</t>
+          <t>Candidate Tayyaba Gull has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -978,7 +978,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Candidate 09_MUHAMMAD_ABUBAKAR has no books listed in their CV.</t>
+          <t>Candidate Muhammad Abubakar has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Candidate 10_MUHAMMAD_EHATISHAM has no books listed in their CV.</t>
+          <t>Candidate Muhammad Ehatisham has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Candidate 11_WAQAS_AMIN has no books listed in their CV.</t>
+          <t>Candidate Waqas Amin has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Candidate 12_SYED_TAMOORULHASSAN has no books listed in their CV.</t>
+          <t>Candidate SYED TAMOORULHASSAN has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1194,7 +1194,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Candidate 13_MANZOOR_ELLAHI has no books listed in their CV.</t>
+          <t>Candidate Manzoor Ellahi has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Candidate 14_SAROSH_TAHIR has no books listed in their CV.</t>
+          <t>Candidate Sarosh Tahir has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Candidate 15_M_USMAN_ABBASI has no books listed in their CV.</t>
+          <t>Candidate M. Usman Abbasi has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1356,7 +1356,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Candidate 16_MUZZAMIL_GHAFFAR has no books listed in their CV.</t>
+          <t>Candidate Muzzamil Ghaffar has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Candidate 17_SUHAIL_ASGHAR has no books listed in their CV.</t>
+          <t>Candidate Suhail Asghar Qureshi has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Candidate 18_MUHAMMAD_AMJAD has no books listed in their CV.</t>
+          <t>Candidate Muhammad Amjad has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Candidate 19_ASIM_MASOOD has no books listed in their CV.</t>
+          <t>Candidate Asim Masood has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1572,7 +1572,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Candidate 20_SYED_FASIH_ALI has no books listed in their CV.</t>
+          <t>Candidate Syed Fasih Ali has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Candidate 21_SAMAN_FATIMA has no books listed in their CV.</t>
+          <t>Candidate Saman Fatima has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1680,7 +1680,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Candidate 22_ZEESHAN has no books listed in their CV.</t>
+          <t>Candidate Zeeshan has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Candidate 23_WAQAS_TARIQ_TOOR has no books listed in their CV.</t>
+          <t>Candidate Waqas Tariq Toor has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -1788,7 +1788,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Candidate 24_AHMED_NAEEM has no books listed in their CV.</t>
+          <t>Candidate Ahmed Naeem has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Candidate 25_MUHAMMAD_ADEEL_ALTAF has no books listed in their CV.</t>
+          <t>Candidate MUHAMMAD ADEEL ALTAF has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -1896,7 +1896,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Candidate 26_AAMINA_AKBAR has no books listed in their CV.</t>
+          <t>Candidate Aamina Akbar has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -1950,7 +1950,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Candidate 27_SHAHEER has no books listed in their CV.</t>
+          <t>Candidate Shaheer has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2004,7 +2004,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Candidate 28_IDRIS_KHAN has no books listed in their CV.</t>
+          <t>Candidate Idris Khan has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2058,7 +2058,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Candidate 29_MUHAMMAD_SARMAD_TARIQ has no books listed in their CV.</t>
+          <t>Candidate Muhammad Sarmad Tariq has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>Candidate 30_FAHD_SIKANDAR_KHAN has no books listed in their CV.</t>
+          <t>Candidate Fahd Sikandar Khan has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2166,7 +2166,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Candidate 31_USMAN_MASUD has no books listed in their CV.</t>
+          <t>Candidate Usman Masud has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2220,7 +2220,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Candidate 32_QAISAR_HUSSAIN_ALVI has no books listed in their CV.</t>
+          <t>Candidate Qaisar Hussain Alvi has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2274,7 +2274,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>Candidate 33_QAMAR_ABBAS has no books listed in their CV.</t>
+          <t>Candidate Qamar Abbas has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2328,7 +2328,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Candidate 34_SHAHZAD has no books listed in their CV.</t>
+          <t>Candidate Shahzad has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -2382,7 +2382,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Candidate 35_MATIULLAH_AHSAN has no books listed in their CV.</t>
+          <t>Candidate Matiullah Ahsan has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -2436,7 +2436,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Candidate 36_SAMANA_BATOOL has no books listed in their CV.</t>
+          <t>Candidate Samana Batool has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2490,7 +2490,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>Candidate 37_SANIA_GUL has no books listed in their CV.</t>
+          <t>Candidate Sania Gul has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Candidate 38_MUHAMMAD_MUSADIQ has no books listed in their CV.</t>
+          <t>Candidate Muhammad Musadiq Ahmed has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>Candidate 39_MUHAMMAD_SAQIB has no books listed in their CV.</t>
+          <t>Candidate Muhammad Saqib has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -2652,7 +2652,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>Candidate 40_ABDUR_REHMAN has no books listed in their CV.</t>
+          <t>Candidate Abdur Rehman has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -2706,7 +2706,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>Candidate 41_MUHAMMAD_AQEEL has no books listed in their CV.</t>
+          <t>Candidate Muhammad Aqeel has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -2760,7 +2760,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>Candidate 42_SAQIB_JAMIL has no books listed in their CV.</t>
+          <t>Candidate Saqib Jamil has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>Candidate 43_AMMARA_NASIM has no books listed in their CV.</t>
+          <t>Candidate Ammara Nasim has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">

</xml_diff>

<commit_message>
Fix CV upload pipeline, LLM rate limit handling, bulk PDF processing, and JD evaluation rules (PhD boost, skill equivalences, 0-skill zero-tolerance rule)
</commit_message>
<xml_diff>
--- a/data/analysis/book_aggregates.xlsx
+++ b/data/analysis/book_aggregates.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N44"/>
+  <dimension ref="A1:N46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -990,12 +990,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>10_MUHAMMAD_EHATISHAM</t>
+          <t>09_SANA_FATIMA_RIZVI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Muhammad Ehatisham</t>
+          <t>Sana Fatima Rizvi</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Candidate Muhammad Ehatisham has no books authored or listed in their CV.</t>
+          <t>Candidate Sana Fatima Rizvi has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1044,12 +1044,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>11_WAQAS_AMIN</t>
+          <t>10_MUHAMMAD_EHATISHAM</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Waqas Amin</t>
+          <t>Muhammad Ehatisham</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Candidate Waqas Amin has no books authored or listed in their CV.</t>
+          <t>Candidate Muhammad Ehatisham has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1098,12 +1098,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12_SYED_TAMOORULHASSAN</t>
+          <t>11_WAQAS_AMIN</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SYED TAMOORULHASSAN</t>
+          <t>Waqas Amin</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Candidate SYED TAMOORULHASSAN has no books authored or listed in their CV.</t>
+          <t>Candidate Waqas Amin has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1152,12 +1152,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>13_MANZOOR_ELLAHI</t>
+          <t>12_SYED_TAMOORULHASSAN</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Manzoor Ellahi</t>
+          <t>SYED TAMOORULHASSAN</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1194,7 +1194,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Candidate Manzoor Ellahi has no books authored or listed in their CV.</t>
+          <t>Candidate SYED TAMOORULHASSAN has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1206,12 +1206,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>14_SAROSH_TAHIR</t>
+          <t>13_MANZOOR_ELLAHI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Sarosh Tahir</t>
+          <t>Manzoor Ellahi</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Candidate Sarosh Tahir has no books authored or listed in their CV.</t>
+          <t>Candidate Manzoor Ellahi has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1260,12 +1260,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>15_M_USMAN_ABBASI</t>
+          <t>14_SAROSH_TAHIR</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>M. Usman Abbasi</t>
+          <t>Sarosh Tahir</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Candidate M. Usman Abbasi has no books authored or listed in their CV.</t>
+          <t>Candidate Sarosh Tahir has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1314,12 +1314,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>16_MUZZAMIL_GHAFFAR</t>
+          <t>15_M_USMAN_ABBASI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Muzzamil Ghaffar</t>
+          <t>M. Usman Abbasi</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1356,7 +1356,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Candidate Muzzamil Ghaffar has no books authored or listed in their CV.</t>
+          <t>Candidate M. Usman Abbasi has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1368,12 +1368,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>17_SUHAIL_ASGHAR</t>
+          <t>16_MUZZAMIL_GHAFFAR</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Suhail Asghar Qureshi</t>
+          <t>Muzzamil Ghaffar</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Candidate Suhail Asghar Qureshi has no books authored or listed in their CV.</t>
+          <t>Candidate Muzzamil Ghaffar has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1422,12 +1422,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>18_MUHAMMAD_AMJAD</t>
+          <t>17_SUHAIL_ASGHAR</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Muhammad Amjad</t>
+          <t>Suhail Asghar Qureshi</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Candidate Muhammad Amjad has no books authored or listed in their CV.</t>
+          <t>Candidate Suhail Asghar Qureshi has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1476,12 +1476,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>19_ASIM_MASOOD</t>
+          <t>18_MUHAMMAD_AMJAD</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Asim Masood</t>
+          <t>Muhammad Amjad</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Candidate Asim Masood has no books authored or listed in their CV.</t>
+          <t>Candidate Muhammad Amjad has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1530,12 +1530,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>20_SYED_FASIH_ALI</t>
+          <t>19_ASIM_MASOOD</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Syed Fasih Ali</t>
+          <t>Asim Masood</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -1572,7 +1572,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Candidate Syed Fasih Ali has no books authored or listed in their CV.</t>
+          <t>Candidate Asim Masood has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1584,12 +1584,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>21_SAMAN_FATIMA</t>
+          <t>20_SYED_FASIH_ALI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Saman Fatima</t>
+          <t>Syed Fasih Ali</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Candidate Saman Fatima has no books authored or listed in their CV.</t>
+          <t>Candidate Syed Fasih Ali has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1638,12 +1638,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>22_ZEESHAN</t>
+          <t>21_SAMAN_FATIMA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Zeeshan</t>
+          <t>Saman Fatima</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -1680,7 +1680,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Candidate Zeeshan has no books authored or listed in their CV.</t>
+          <t>Candidate Saman Fatima has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -1692,12 +1692,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>23_WAQAS_TARIQ_TOOR</t>
+          <t>22_ZEESHAN</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Waqas Tariq Toor</t>
+          <t>Zeeshan</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Candidate Waqas Tariq Toor has no books authored or listed in their CV.</t>
+          <t>Candidate Zeeshan has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -1746,12 +1746,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>24_AHMED_NAEEM</t>
+          <t>23_WAQAS_TARIQ_TOOR</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Ahmed Naeem</t>
+          <t>Waqas Tariq Toor</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -1788,7 +1788,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Candidate Ahmed Naeem has no books authored or listed in their CV.</t>
+          <t>Candidate Waqas Tariq Toor has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -1800,12 +1800,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>25_MUHAMMAD_ADEEL_ALTAF</t>
+          <t>24_AHMED_NAEEM</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>MUHAMMAD ADEEL ALTAF</t>
+          <t>Ahmed Naeem</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Candidate MUHAMMAD ADEEL ALTAF has no books authored or listed in their CV.</t>
+          <t>Candidate Ahmed Naeem has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -1854,12 +1854,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>26_AAMINA_AKBAR</t>
+          <t>25_MUHAMMAD_ADEEL_ALTAF</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Aamina Akbar</t>
+          <t>MUHAMMAD ADEEL ALTAF</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -1896,7 +1896,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Candidate Aamina Akbar has no books authored or listed in their CV.</t>
+          <t>Candidate MUHAMMAD ADEEL ALTAF has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -1908,12 +1908,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>27_SHAHEER</t>
+          <t>26_AAMINA_AKBAR</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Shaheer</t>
+          <t>Aamina Akbar</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -1950,7 +1950,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Candidate Shaheer has no books authored or listed in their CV.</t>
+          <t>Candidate Aamina Akbar has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -1962,12 +1962,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>28_IDRIS_KHAN</t>
+          <t>27_SHAHEER</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Idris Khan</t>
+          <t>Shaheer</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -2004,7 +2004,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Candidate Idris Khan has no books authored or listed in their CV.</t>
+          <t>Candidate Shaheer has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2016,12 +2016,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>29_MUHAMMAD_SARMAD_TARIQ</t>
+          <t>28_IDRIS_KHAN</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Muhammad Sarmad Tariq</t>
+          <t>Idris Khan</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -2058,7 +2058,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Candidate Muhammad Sarmad Tariq has no books authored or listed in their CV.</t>
+          <t>Candidate Idris Khan has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2070,12 +2070,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>30_FAHD_SIKANDAR_KHAN</t>
+          <t>29_MUHAMMAD_SARMAD_TARIQ</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Fahd Sikandar Khan</t>
+          <t>Muhammad Sarmad Tariq</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>Candidate Fahd Sikandar Khan has no books authored or listed in their CV.</t>
+          <t>Candidate Muhammad Sarmad Tariq has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2124,12 +2124,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>31_USMAN_MASUD</t>
+          <t>30_FAHD_SIKANDAR_KHAN</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Usman Masud</t>
+          <t>Fahd Sikandar Khan</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -2166,7 +2166,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Candidate Usman Masud has no books authored or listed in their CV.</t>
+          <t>Candidate Fahd Sikandar Khan has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2178,12 +2178,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>32_QAISAR_HUSSAIN_ALVI</t>
+          <t>31_USMAN_MASUD</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Qaisar Hussain Alvi</t>
+          <t>Usman Masud</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -2220,7 +2220,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Candidate Qaisar Hussain Alvi has no books authored or listed in their CV.</t>
+          <t>Candidate Usman Masud has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2232,12 +2232,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>33_QAMAR_ABBAS</t>
+          <t>32_QAISAR_HUSSAIN_ALVI</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Qamar Abbas</t>
+          <t>Qaisar Hussain Alvi</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -2274,7 +2274,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>Candidate Qamar Abbas has no books authored or listed in their CV.</t>
+          <t>Candidate Qaisar Hussain Alvi has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2286,12 +2286,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>34_SHAHZAD</t>
+          <t>33_QAMAR_ABBAS</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Shahzad</t>
+          <t>Qamar Abbas</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -2328,7 +2328,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Candidate Shahzad has no books authored or listed in their CV.</t>
+          <t>Candidate Qamar Abbas has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -2340,12 +2340,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>35_MATIULLAH_AHSAN</t>
+          <t>34_SHAHZAD</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Matiullah Ahsan</t>
+          <t>Shahzad</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -2382,7 +2382,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Candidate Matiullah Ahsan has no books authored or listed in their CV.</t>
+          <t>Candidate Shahzad has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -2394,12 +2394,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>36_SAMANA_BATOOL</t>
+          <t>35_MATIULLAH_AHSAN</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Samana Batool</t>
+          <t>Matiullah Ahsan</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -2436,7 +2436,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Candidate Samana Batool has no books authored or listed in their CV.</t>
+          <t>Candidate Matiullah Ahsan has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2448,12 +2448,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>37_SANIA_GUL</t>
+          <t>36_SAMANA_BATOOL</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Sania Gul</t>
+          <t>Samana Batool</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -2490,7 +2490,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>Candidate Sania Gul has no books authored or listed in their CV.</t>
+          <t>Candidate Samana Batool has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2502,12 +2502,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>38_MUHAMMAD_MUSADIQ</t>
+          <t>37_SANIA_GUL</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Muhammad Musadiq Ahmed</t>
+          <t>Sania Gul</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Candidate Muhammad Musadiq Ahmed has no books authored or listed in their CV.</t>
+          <t>Candidate Sania Gul has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -2556,12 +2556,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>39_MUHAMMAD_SAQIB</t>
+          <t>38_MUHAMMAD_MUSADIQ</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Muhammad Saqib</t>
+          <t>Muhammad Musadiq Ahmed</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>Candidate Muhammad Saqib has no books authored or listed in their CV.</t>
+          <t>Candidate Muhammad Musadiq Ahmed has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -2610,12 +2610,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>40_ABDUR_REHMAN</t>
+          <t>39_MUHAMMAD_SAQIB</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Abdur Rehman</t>
+          <t>Muhammad Saqib</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -2652,7 +2652,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>Candidate Abdur Rehman has no books authored or listed in their CV.</t>
+          <t>Candidate Muhammad Saqib has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -2664,12 +2664,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>41_MUHAMMAD_AQEEL</t>
+          <t>40_ABDUR_REHMAN</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Muhammad Aqeel</t>
+          <t>Abdur Rehman</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -2706,7 +2706,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>Candidate Muhammad Aqeel has no books authored or listed in their CV.</t>
+          <t>Candidate Abdur Rehman has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -2718,12 +2718,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>42_SAQIB_JAMIL</t>
+          <t>41_MUHAMMAD_AQEEL</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Saqib Jamil</t>
+          <t>Muhammad Aqeel</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -2760,7 +2760,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>Candidate Saqib Jamil has no books authored or listed in their CV.</t>
+          <t>Candidate Muhammad Aqeel has no books authored or listed in their CV.</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -2772,52 +2772,160 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>42_SAQIB_JAMIL</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Saqib Jamil</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>No Books Listed</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>Candidate Saqib Jamil has no books authored or listed in their CV.</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>No Books Listed</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>43_AMMARA_NASIM</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>Ammara Nasim</t>
         </is>
       </c>
-      <c r="C44" t="n">
-        <v>0</v>
-      </c>
-      <c r="D44" t="n">
-        <v>0</v>
-      </c>
-      <c r="E44" t="n">
-        <v>0</v>
-      </c>
-      <c r="F44" t="n">
-        <v>0</v>
-      </c>
-      <c r="G44" t="n">
-        <v>0</v>
-      </c>
-      <c r="H44" t="n">
-        <v>0</v>
-      </c>
-      <c r="I44" t="n">
-        <v>0</v>
-      </c>
-      <c r="J44" t="n">
-        <v>0</v>
-      </c>
-      <c r="K44" t="n">
-        <v>0</v>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>No Books Listed</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
+      <c r="C45" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>No Books Listed</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
         <is>
           <t>Candidate Ammara Nasim has no books authored or listed in their CV.</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr">
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>No Books Listed</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Muhammad_Dawood_Rizwan_CV</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>No Books Listed</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>Candidate nan has no books authored or listed in their CV.</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
         <is>
           <t>No Books Listed</t>
         </is>

</xml_diff>